<commit_message>
Add DDG Grand-Block Outsourcing tab to the module-cost workbook
New guide tab (6 -> 7 sheets): the 22 SAM/FSRS subaward actions whose SOW
text explicitly names a grand block - Gulf Copper $31.6M, BAE Jacksonville
$17.7M (GB B15), Eastern Shipbuilding $5.6M; $55.0M then-year net, DDG 137
= $49.2M across ~8 named blocks - with the DDG 137 per-block split, yard
roll-up, and a live cost anchor against the Module Cost per-grand-block
allocation (largest block ~24% of the fully-burdened even split; a floor,
not a make-vs-buy ratio). SAM-to-Module Bridge gains a §5 explicit-text
cross-reference; validate_workbook.py gains three tie-outs (3-yard total,
DDG 137 partition, anchor = ship BC / 21). Verified: build + LibreOffice
recalc clean, all checks OK.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/distributed_shipbuilding/ddg_module_cost/20260625_DDG-51 Module Cost_vS.xlsx
+++ b/projects/distributed_shipbuilding/ddg_module_cost/20260625_DDG-51 Module Cost_vS.xlsx
@@ -9,9 +9,10 @@
     <sheet name="Module Cost" sheetId="1" r:id="rId1"/>
     <sheet name="Structural Hierarchy" sheetId="2" r:id="rId2"/>
     <sheet name="SAM-to-Module Bridge Notes" sheetId="3" r:id="rId3"/>
-    <sheet name="Assumptions" sheetId="4" r:id="rId4"/>
-    <sheet name="Ship Cost Basis" sheetId="5" r:id="rId5"/>
-    <sheet name="Outfit Context" sheetId="6" r:id="rId6"/>
+    <sheet name="DDG Grand-Block Outsourcing" sheetId="4" r:id="rId4"/>
+    <sheet name="Assumptions" sheetId="5" r:id="rId5"/>
+    <sheet name="Ship Cost Basis" sheetId="6" r:id="rId6"/>
+    <sheet name="Outfit Context" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1323,11 +1324,644 @@
         </is>
       </c>
     </row>
+    <row r="42" outlineLevel="2"/>
+    <row r="43" outlineLevel="2"/>
+    <row r="44" outlineLevel="1">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">§5 - The explicit-text case: grand-block outsourcing</t>
+        </is>
+      </c>
+      <c r="C44" s="9"/>
+    </row>
+    <row r="45" outlineLevel="2">
+      <c r="B45" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Where the §2 / §3 rule actually fires - subawards that DO name the block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" outlineLevel="2"/>
+    <row r="47" outlineLevel="2">
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What it is</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the FY2018-22 multi-year buy, HII outsourced fabrication of whole grand blocks to three yards (Gulf Copper, BAE Jacksonville, Eastern Shipbuilding). Their SOW text names the block - "GB B15", "GB A16 &amp; A21", "C15GB", "GRAND BLOCK" - so these subawards attribute to a physical grand block on explicit text, exactly as §3 permits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" outlineLevel="2">
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why it stays rare</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is the visible tail of make-vs-buy: only OUTSOURCED blocks generate a block-named subaward. In-house blocks never enter the subaward corpus, so this lens sees outsourced fabrication only, not the full block population.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" outlineLevel="2">
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The DDG Grand-Block Outsourcing tab - the verbatim evidence, the per-block split for DDG 137, and a first bottom-up check of outsourced fabrication against the Module Cost per-grand-block allocation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF2C5E5E"/>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="10" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="2.2109375" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="56" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DDG Grand-Block Outsourcing</t>
+        </is>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+    </row>
+    <row r="3" outlineLevel="1">
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outsourced grand-block fabrication - the subawards that name a physical block</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" outlineLevel="1"/>
+    <row r="5" outlineLevel="1"/>
+    <row r="6" outlineLevel="1">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">§1 - Direct evidence: subawards that name a grand block</t>
+        </is>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" outlineLevel="2"/>
+    <row r="8" outlineLevel="2">
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For the FY2018-22 multi-year buy, three yards fabricated whole grand blocks under subaward. Unlike routine component supply, their statement-of-work descriptions name the block - the rare explicit-text case the SAM-to-Module Bridge Notes tab (§2-§3) calls for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" outlineLevel="2"/>
+    <row r="10" outlineLevel="2">
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (GB B15)"  -  BAE Systems Jacksonville, $17.7M (2 actions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" outlineLevel="2">
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (GB A16 &amp; A21)"  -  Gulf Copper, $5.4M</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" outlineLevel="2">
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (GB B43 &amp; B13)"  -  Gulf Copper, $5.0M</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" outlineLevel="2">
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 C15GB UNIT OUTSOURCING"  -  Eastern Shipbuilding, $5.3M</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" outlineLevel="2">
+      <c r="B14" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 139 SOW UNIT OUTSOURCING (GB D52)"  -  Gulf Copper, $4.7M</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" outlineLevel="2">
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 GRAND BLOCK"  -  Gulf Copper, $0.7M</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" outlineLevel="2"/>
+    <row r="17" outlineLevel="2">
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 yards  |  22 subaward actions  |  hulls DDG 135 / 137 / 139  |  $55.0M then-year (net of credits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" outlineLevel="2"/>
+    <row r="19" outlineLevel="2"/>
+    <row r="20" outlineLevel="1">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">§2 - DDG 137 by grand block (the full-coverage hull)</t>
+        </is>
+      </c>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" outlineLevel="2"/>
+    <row r="22" outlineLevel="2">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grand block</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yard</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Net $M</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description (verbatim)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" outlineLevel="2">
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B15</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAE Jax</t>
+        </is>
+      </c>
+      <c r="D23" s="5">
+        <v>17.72</v>
+      </c>
+      <c r="E23" s="45">
+        <v>2</v>
+      </c>
+      <c r="F23" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (GB B15)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" outlineLevel="2">
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D52</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulf Copper</t>
+        </is>
+      </c>
+      <c r="D24" s="5">
+        <v>10.88</v>
+      </c>
+      <c r="E24" s="45">
+        <v>5</v>
+      </c>
+      <c r="F24" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (D52)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" outlineLevel="2">
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A16 &amp; A21</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulf Copper</t>
+        </is>
+      </c>
+      <c r="D25" s="5">
+        <v>5.37</v>
+      </c>
+      <c r="E25" s="45">
+        <v>4</v>
+      </c>
+      <c r="F25" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (GB A16 &amp; A21)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" outlineLevel="2">
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C15</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eastern</t>
+        </is>
+      </c>
+      <c r="D26" s="5">
+        <v>5.31</v>
+      </c>
+      <c r="E26" s="45">
+        <v>1</v>
+      </c>
+      <c r="F26" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 C15GB UNIT OUTSOURCING"</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" outlineLevel="2">
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B43 &amp; B13</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulf Copper</t>
+        </is>
+      </c>
+      <c r="D27" s="5">
+        <v>5.01</v>
+      </c>
+      <c r="E27" s="45">
+        <v>1</v>
+      </c>
+      <c r="F27" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (GB B43 &amp; B13)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" outlineLevel="2">
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D41 / D42</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulf Copper</t>
+        </is>
+      </c>
+      <c r="D28" s="5">
+        <v>2.51</v>
+      </c>
+      <c r="E28" s="45">
+        <v>3</v>
+      </c>
+      <c r="F28" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (D41/D42)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" outlineLevel="2">
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D11 / D21 / D31</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulf Copper</t>
+        </is>
+      </c>
+      <c r="D29" s="5">
+        <v>1.68</v>
+      </c>
+      <c r="E29" s="45">
+        <v>1</v>
+      </c>
+      <c r="F29" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 SOW UNIT OUTSOURCING (D11, D21, D31)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" outlineLevel="2">
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(unlabeled)</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulf Copper</t>
+        </is>
+      </c>
+      <c r="D30" s="5">
+        <v>0.74</v>
+      </c>
+      <c r="E30" s="45">
+        <v>1</v>
+      </c>
+      <c r="F30" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"DDG 137 GRAND BLOCK"</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" outlineLevel="2">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DDG 137 grand-block total</t>
+        </is>
+      </c>
+      <c r="C31" s="16"/>
+      <c r="D31" s="13">
+        <f>SUM(D23:D30)</f>
+      </c>
+      <c r="E31" s="47">
+        <f>SUM(E23:E30)</f>
+      </c>
+      <c r="F31" s="16"/>
+    </row>
+    <row r="32" outlineLevel="2">
+      <c r="B32" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D52 is net of a -$7.2M Oct-2025 rescope (partial deobligation of an $8.2M award); the (unlabeled) row's SOW reads only "GRAND BLOCK".</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" outlineLevel="2"/>
+    <row r="34" outlineLevel="2"/>
+    <row r="35" outlineLevel="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">§3 - By yard (all hulls, then-year $ net of credits)</t>
+        </is>
+      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+    </row>
+    <row r="36" outlineLevel="2"/>
+    <row r="37" outlineLevel="2">
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yard</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Net $M</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hulls</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" outlineLevel="2">
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulf Copper &amp; Mfg</t>
+        </is>
+      </c>
+      <c r="C38" s="5">
+        <v>31.59</v>
+      </c>
+      <c r="D38" s="45">
+        <v>17</v>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">135, 137, 139</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" outlineLevel="2">
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAE Systems Jacksonville</t>
+        </is>
+      </c>
+      <c r="C39" s="5">
+        <v>17.72</v>
+      </c>
+      <c r="D39" s="45">
+        <v>2</v>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">137</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" outlineLevel="2">
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eastern Shipbuilding</t>
+        </is>
+      </c>
+      <c r="C40" s="5">
+        <v>5.65</v>
+      </c>
+      <c r="D40" s="45">
+        <v>3</v>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">135, 137, 139</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" outlineLevel="2">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grand-block outsourcing, 3 yards</t>
+        </is>
+      </c>
+      <c r="C41" s="13">
+        <f>SUM(C38:C40)</f>
+      </c>
+      <c r="D41" s="47">
+        <f>SUM(D38:D40)</f>
+      </c>
+      <c r="E41" s="16"/>
+    </row>
+    <row r="42" outlineLevel="2">
+      <c r="B42" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">By hull: DDG 137 $49.2M · DDG 139 $4.8M · DDG 135 $0.9M. All on the FY2018-22 block-buy; all read in-build (post-keel) on the SAM timing axis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" outlineLevel="2"/>
+    <row r="44" outlineLevel="2"/>
+    <row r="45" outlineLevel="1">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">§4 - Cost anchor: outsourced fabrication vs the model</t>
+        </is>
+      </c>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+    </row>
+    <row r="46" outlineLevel="2"/>
+    <row r="47" outlineLevel="2">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measure</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" outlineLevel="2">
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model allocation per grand block (even split)</t>
+        </is>
+      </c>
+      <c r="C48" s="11">
+        <f>'Assumptions'!C10/'Assumptions'!C17</f>
+      </c>
+    </row>
+    <row r="49" outlineLevel="2">
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Largest outsourced block (BAE, GB B15)</t>
+        </is>
+      </c>
+      <c r="C49" s="5">
+        <v>17.72</v>
+      </c>
+    </row>
+    <row r="50" outlineLevel="2">
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  as share of the model per-block allocation</t>
+        </is>
+      </c>
+      <c r="C50" s="6">
+        <f>C49/C48</f>
+      </c>
+    </row>
+    <row r="51" outlineLevel="2"/>
+    <row r="52" outlineLevel="2">
+      <c r="B52" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outsourced work is bare structural fabrication (steel + welding) of a grand block - a FLOOR on that block's cost. Observed per block runs ~$1.7M-$17.7M, roughly 2-24% of the model's fully-burdened Basic-Construction allocation; erection, outfitting, systems integration and test stay at the prime yard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" outlineLevel="2">
+      <c r="B53" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The model figure is an even split; the outsourced hull-structure blocks (A/B/C/D zones) are likely below-average-cost blocks, so read this as an order-of-magnitude band, not a precise ratio. Then-year $ vs the model's const FY2026 $ differ ~2-4% here - immaterial to the band.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" outlineLevel="2"/>
+    <row r="55" outlineLevel="2"/>
+    <row r="56" outlineLevel="2">
+      <c r="B56" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source: SAM.gov FSRS first-tier subaward records, DDG-51 program; grand-block rows are those whose description explicitly names a PWBS block / zone (GB A16, GB B15, C15GB, D52, ...). Then-year $M, net of credits. Captured 2026-07-01.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF556B2F"/>
@@ -1556,7 +2190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF203864"/>
@@ -2169,7 +2803,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF203864"/>

</xml_diff>